<commit_message>
Phase 3 follow-up: model additions, single metric definitions, rule detail
- fact_activity: officer_code, quality_flag (ok/info/warning), on_time;
  fact_indicator_result: officer_code, quality_flag on the same scheme;
  dim_location: location_level, with a model check and test that no
  aggregation mixes village and district rows
- dim_beneficiary.pending_duplicate_review (32 people); 1,509 vs 1,500
  explained (9 people split by name-only matches awaiting review)
- config/dq_metrics.yaml: one definition per measure, used by the rules,
  the report, the warehouse and the scorer (timeliness 88.8% everywhere)
- dq_results.dimension_impact and dq_rule_results_by_file
- Optional officer code column in the beneficiary register template
- 224 tests passing

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/beneficiary_register_template.xlsx
+++ b/templates/beneficiary_register_template.xlsx
@@ -170,6 +170,11 @@
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Surname first, then given names</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional: the field officer who registered this person</t>
       </text>
     </comment>
   </commentList>
@@ -517,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2001"/>
+  <dimension ref="A1:O2001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -534,6 +539,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -607,6 +613,11 @@
           <t>Registration date</t>
         </is>
       </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Officer code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n"/>
@@ -20609,9 +20620,9 @@
       <c r="N2001" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation sqref="C2:C2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please pick a value from the list." type="list">
-      <formula1>=Lists!$D$2:$D$3</formula1>
+      <formula1>=Lists!$E$2:$E$3</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please type a whole number (0 or more)." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
@@ -20620,17 +20631,20 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please pick a value from the list." type="list">
-      <formula1>=Lists!$E$2:$E$3</formula1>
+      <formula1>=Lists!$F$2:$F$3</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please pick a value from the list." type="list">
       <formula1>=Lists!$B$2:$B$31</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please pick a value from the list." type="list">
-      <formula1>=Lists!$C$2:$C$6</formula1>
+      <formula1>=Lists!$D$2:$D$6</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please type a date, for example 12/03/2024." type="date" operator="between">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
+    </dataValidation>
+    <dataValidation sqref="O2:O2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Please pick a value from the list." type="list">
+      <formula1>=Lists!$C$2:$C$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -30695,7 +30709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30711,15 +30725,20 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>officers</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
+          <t>projects</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>yes_no</t>
         </is>
@@ -30738,15 +30757,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Community Water Access</t>
+          <t>FO01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Community Water Access</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -30765,15 +30789,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Household and School Sanitation</t>
+          <t>FO02</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Household and School Sanitation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -30792,6 +30821,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>FO03</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Hygiene Behaviour Change</t>
         </is>
       </c>
@@ -30809,6 +30843,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>FO04</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Climate-Smart Farmer Field Schools</t>
         </is>
       </c>
@@ -30826,6 +30865,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>DE01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Solar Irrigation and Cooperatives</t>
         </is>
       </c>

</xml_diff>